<commit_message>
Mise à jour portfolio: ajout descriptions projets PPE, modifications stages, suppression tableau synthèse
</commit_message>
<xml_diff>
--- a/a copier BTS SIO 2026 - Tableau de synthèse - Epreuve E4.xlsx
+++ b/a copier BTS SIO 2026 - Tableau de synthèse - Epreuve E4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c8c2de6d2e26ef7/Desktop/Portfolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="59" documentId="8_{C7F3F2AB-635F-4E44-869C-52D6CF67124C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87A53D48-0AC5-4780-90ED-511E117AFBBC}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="8_{C7F3F2AB-635F-4E44-869C-52D6CF67124C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{426C544C-19CC-4798-9AB3-D01901A09E65}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -63,9 +63,6 @@
     <t xml:space="preserve">▣ </t>
   </si>
   <si>
-    <t xml:space="preserve">Adresse URL du portfolio : </t>
-  </si>
-  <si>
     <t>Compétences mises en œuvre
 Réalisations professionnelles
 (intitulé et liste des documents et productions associés)</t>
@@ -207,6 +204,9 @@
   </si>
   <si>
     <t>du 5/01/26 au 5/02/26</t>
+  </si>
+  <si>
+    <t>Adresse URL du portfolio : https://nefakul.github.io/Portfolio/</t>
   </si>
 </sst>
 </file>
@@ -258,12 +258,6 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
     </font>
     <font>
       <b/>
@@ -319,6 +313,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -723,10 +724,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -735,8 +736,14 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -744,46 +751,40 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -792,31 +793,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
@@ -825,9 +826,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -841,11 +839,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="16" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="15" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1079,40 +1080,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="48" t="s">
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="49"/>
+      <c r="H1" s="48"/>
     </row>
     <row r="2" spans="1:13" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
     </row>
     <row r="3" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="50" t="s">
-        <v>25</v>
+      <c r="A3" s="49" t="s">
+        <v>24</v>
       </c>
       <c r="B3" s="38"/>
       <c r="C3" s="38"/>
       <c r="D3" s="38"/>
-      <c r="E3" s="51"/>
-      <c r="F3" s="52" t="s">
+      <c r="E3" s="50"/>
+      <c r="F3" s="51" t="s">
         <v>3</v>
       </c>
       <c r="G3" s="38"/>
@@ -1123,7 +1124,7 @@
     </row>
     <row r="4" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="43" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B4" s="41"/>
       <c r="C4" s="41"/>
@@ -1136,7 +1137,7 @@
         <v>5</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>6</v>
@@ -1146,68 +1147,68 @@
       </c>
     </row>
     <row r="5" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="45" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="46"/>
-      <c r="C5" s="46"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="46"/>
-      <c r="F5" s="46"/>
-      <c r="G5" s="46"/>
-      <c r="H5" s="47"/>
+      <c r="A5" s="54" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="46"/>
     </row>
     <row r="6" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="33" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="C6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="F6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="G6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="H6" s="8" t="s">
         <v>15</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="324.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="34"/>
       <c r="B7" s="36"/>
       <c r="C7" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="E7" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="F7" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="G7" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="H7" s="10" t="s">
         <v>21</v>
-      </c>
-      <c r="H7" s="10" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="37" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" s="38"/>
       <c r="C8" s="38"/>
@@ -1219,70 +1220,70 @@
     </row>
     <row r="9" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="12"/>
       <c r="E9" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H9" s="13"/>
     </row>
     <row r="10" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E10" s="12"/>
       <c r="F10" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H10" s="13"/>
     </row>
     <row r="11" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E11" s="12"/>
       <c r="F11" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H11" s="13"/>
     </row>
     <row r="12" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="24" t="s">
         <v>40</v>
-      </c>
-      <c r="B12" s="24" t="s">
-        <v>41</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12"/>
@@ -1290,7 +1291,7 @@
       <c r="F12" s="12"/>
       <c r="G12" s="12"/>
       <c r="H12" s="13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1355,7 +1356,7 @@
     </row>
     <row r="19" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="40" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B19" s="41"/>
       <c r="C19" s="41"/>
@@ -1367,63 +1368,63 @@
     </row>
     <row r="20" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="B20" s="26" t="s">
-        <v>36</v>
-      </c>
       <c r="C20" s="30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D20" s="30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E20" s="30"/>
       <c r="F20" s="30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G20" s="30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H20" s="32"/>
     </row>
     <row r="21" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="31" t="s">
-        <v>42</v>
-      </c>
-      <c r="B21" s="53" t="s">
-        <v>37</v>
+        <v>41</v>
+      </c>
+      <c r="B21" s="52" t="s">
+        <v>36</v>
       </c>
       <c r="C21" s="14"/>
       <c r="D21" s="30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E21" s="14"/>
       <c r="F21" s="14"/>
       <c r="G21" s="30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H21" s="32" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C22" s="30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D22" s="30"/>
       <c r="E22" s="14"/>
       <c r="F22" s="30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G22" s="30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H22" s="15"/>
     </row>
@@ -1469,7 +1470,7 @@
     </row>
     <row r="27" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="40" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B27" s="41"/>
       <c r="C27" s="41"/>
@@ -1481,28 +1482,28 @@
     </row>
     <row r="28" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B28" s="54" t="s">
-        <v>44</v>
+        <v>31</v>
+      </c>
+      <c r="B28" s="53" t="s">
+        <v>43</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F28" s="30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G28" s="30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H28" s="32" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Mise à jour portfolio: veille technologique, section compétences, et modifications de contenu
</commit_message>
<xml_diff>
--- a/a copier BTS SIO 2026 - Tableau de synthèse - Epreuve E4.xlsx
+++ b/a copier BTS SIO 2026 - Tableau de synthèse - Epreuve E4.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c8c2de6d2e26ef7/Desktop/Portfolio/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2c8c2de6d2e26ef7/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="8_{C7F3F2AB-635F-4E44-869C-52D6CF67124C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{426C544C-19CC-4798-9AB3-D01901A09E65}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C7F580AC-3F9E-4371-BE99-FE53C5CA0D8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="51">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -207,6 +207,24 @@
   </si>
   <si>
     <t>Adresse URL du portfolio : https://nefakul.github.io/Portfolio/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projet Cas Lafleur </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projet Veille Technologique </t>
+  </si>
+  <si>
+    <t>PPE Sipèvizion (présentation monitoring)</t>
+  </si>
+  <si>
+    <t>du 05/11/24 au 11/02/25</t>
+  </si>
+  <si>
+    <t>du 05/09/25 au 27/03/26</t>
+  </si>
+  <si>
+    <t>a partir du 18/02/25</t>
   </si>
 </sst>
 </file>
@@ -802,6 +820,12 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="15" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -826,6 +850,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -837,15 +864,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="15" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -863,10 +881,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1080,56 +1094,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="47" t="s">
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="48"/>
+      <c r="H1" s="51"/>
     </row>
     <row r="2" spans="1:13" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
     </row>
     <row r="3" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="49" t="s">
+      <c r="A3" s="52" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="38"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="51" t="s">
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="54" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="38"/>
-      <c r="H3" s="39"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="41"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="44"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="46"/>
       <c r="F4" s="2" t="s">
         <v>4</v>
       </c>
@@ -1147,22 +1161,22 @@
       </c>
     </row>
     <row r="5" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="54" t="s">
+      <c r="A5" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="45"/>
-      <c r="C5" s="45"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="46"/>
+      <c r="B5" s="48"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="48"/>
+      <c r="E5" s="48"/>
+      <c r="F5" s="48"/>
+      <c r="G5" s="48"/>
+      <c r="H5" s="49"/>
     </row>
     <row r="6" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="37" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="7" t="s">
@@ -1185,8 +1199,8 @@
       </c>
     </row>
     <row r="7" spans="1:13" ht="324.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="34"/>
-      <c r="B7" s="36"/>
+      <c r="A7" s="36"/>
+      <c r="B7" s="38"/>
       <c r="C7" s="9" t="s">
         <v>16</v>
       </c>
@@ -1207,16 +1221,16 @@
       </c>
     </row>
     <row r="8" spans="1:13" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="37" t="s">
+      <c r="A8" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="38"/>
-      <c r="C8" s="38"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="38"/>
-      <c r="F8" s="38"/>
-      <c r="G8" s="38"/>
-      <c r="H8" s="39"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="41"/>
     </row>
     <row r="9" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
@@ -1295,34 +1309,60 @@
       </c>
     </row>
     <row r="13" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="11"/>
-      <c r="B13" s="25"/>
+      <c r="A13" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>50</v>
+      </c>
       <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
+      <c r="D13" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="H13" s="13"/>
     </row>
     <row r="14" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="11"/>
-      <c r="B14" s="22"/>
+      <c r="A14" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="22" t="s">
+        <v>49</v>
+      </c>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
       <c r="E14" s="12"/>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
-      <c r="H14" s="13"/>
+      <c r="H14" s="13" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="15" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="11"/>
-      <c r="B15" s="23"/>
+      <c r="A15" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" s="23" t="s">
+        <v>48</v>
+      </c>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
       <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
+      <c r="F15" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="G15" s="12"/>
-      <c r="H15" s="13"/>
+      <c r="H15" s="13" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="16" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="11"/>
@@ -1355,16 +1395,16 @@
       <c r="H18" s="13"/>
     </row>
     <row r="19" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="40" t="s">
+      <c r="A19" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="41"/>
-      <c r="C19" s="41"/>
-      <c r="D19" s="41"/>
-      <c r="E19" s="41"/>
-      <c r="F19" s="41"/>
-      <c r="G19" s="41"/>
-      <c r="H19" s="42"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="43"/>
+      <c r="E19" s="43"/>
+      <c r="F19" s="43"/>
+      <c r="G19" s="43"/>
+      <c r="H19" s="44"/>
     </row>
     <row r="20" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="31" t="s">
@@ -1392,7 +1432,7 @@
       <c r="A21" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="B21" s="52" t="s">
+      <c r="B21" s="33" t="s">
         <v>36</v>
       </c>
       <c r="C21" s="14"/>
@@ -1469,22 +1509,22 @@
       <c r="H26" s="15"/>
     </row>
     <row r="27" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="40" t="s">
+      <c r="A27" s="42" t="s">
         <v>23</v>
       </c>
-      <c r="B27" s="41"/>
-      <c r="C27" s="41"/>
-      <c r="D27" s="41"/>
-      <c r="E27" s="41"/>
-      <c r="F27" s="41"/>
-      <c r="G27" s="41"/>
-      <c r="H27" s="42"/>
+      <c r="B27" s="43"/>
+      <c r="C27" s="43"/>
+      <c r="D27" s="43"/>
+      <c r="E27" s="43"/>
+      <c r="F27" s="43"/>
+      <c r="G27" s="43"/>
+      <c r="H27" s="44"/>
     </row>
     <row r="28" spans="1:8" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="53" t="s">
+      <c r="B28" s="34" t="s">
         <v>43</v>
       </c>
       <c r="C28" s="30" t="s">
@@ -4286,6 +4326,6 @@
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" scale="48" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>